<commit_message>
Weekly report + learning artifacts
</commit_message>
<xml_diff>
--- a/reports/weekly_bvb_model_vs_real_2025-12-12.xlsx
+++ b/reports/weekly_bvb_model_vs_real_2025-12-12.xlsx
@@ -554,36 +554,36 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>BATE.DE</t>
+          <t>AG</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>EU</t>
+          <t>RO</t>
         </is>
       </c>
       <c r="G2" t="n">
         <v>5</v>
       </c>
       <c r="H2" t="n">
-        <v>0.3</v>
+        <v>-1</v>
       </c>
       <c r="I2" t="n">
-        <v>24.82999992370605</v>
+        <v>1.44</v>
       </c>
       <c r="J2" t="n">
-        <v>24.69000053405762</v>
+        <v>1.46</v>
       </c>
       <c r="K2" t="n">
-        <v>-0.5638316152984379</v>
+        <v>1.388888888888884</v>
       </c>
       <c r="L2" t="n">
-        <v>-0.863831615298438</v>
+        <v>2.388888888888884</v>
       </c>
       <c r="M2" t="n">
-        <v>0.863831615298438</v>
-      </c>
-      <c r="N2" t="b">
+        <v>2.388888888888884</v>
+      </c>
+      <c r="N2" t="n">
         <v>0</v>
       </c>
       <c r="O2" t="inlineStr">
@@ -592,15 +592,15 @@
         </is>
       </c>
       <c r="P2" t="n">
-        <v>0.4468980792022068</v>
+        <v>-1</v>
       </c>
       <c r="Q2" t="n">
-        <v>-1.010729694500645</v>
+        <v>2.388888888888884</v>
       </c>
       <c r="R2" t="n">
-        <v>1.010729694500645</v>
-      </c>
-      <c r="S2" t="b">
+        <v>2.388888888888884</v>
+      </c>
+      <c r="S2" t="n">
         <v>0</v>
       </c>
       <c r="T2" t="b">
@@ -624,36 +624,36 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>LHA.DE</t>
+          <t>ALR</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>EU</t>
+          <t>RO</t>
         </is>
       </c>
       <c r="G3" t="n">
         <v>5</v>
       </c>
       <c r="H3" t="n">
-        <v>-0.4</v>
+        <v>0.5</v>
       </c>
       <c r="I3" t="n">
-        <v>8.255999565124512</v>
+        <v>1.51</v>
       </c>
       <c r="J3" t="n">
-        <v>8.465999603271484</v>
+        <v>1.505</v>
       </c>
       <c r="K3" t="n">
-        <v>2.543605247195835</v>
+        <v>-0.3311258278145823</v>
       </c>
       <c r="L3" t="n">
-        <v>2.943605247195835</v>
+        <v>-0.8311258278145823</v>
       </c>
       <c r="M3" t="n">
-        <v>2.943605247195835</v>
-      </c>
-      <c r="N3" t="b">
+        <v>0.8311258278145823</v>
+      </c>
+      <c r="N3" t="n">
         <v>0</v>
       </c>
       <c r="O3" t="inlineStr">
@@ -662,19 +662,19 @@
         </is>
       </c>
       <c r="P3" t="n">
-        <v>0.2432647407719428</v>
+        <v>0.5</v>
       </c>
       <c r="Q3" t="n">
-        <v>2.300340506423892</v>
+        <v>-0.8311258278145823</v>
       </c>
       <c r="R3" t="n">
-        <v>2.300340506423892</v>
-      </c>
-      <c r="S3" t="b">
+        <v>0.8311258278145823</v>
+      </c>
+      <c r="S3" t="n">
         <v>0</v>
       </c>
       <c r="T3" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4">
@@ -694,7 +694,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>AG</t>
+          <t>AQ</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -706,25 +706,25 @@
         <v>5</v>
       </c>
       <c r="H4" t="n">
-        <v>-1</v>
+        <v>0.7</v>
       </c>
       <c r="I4" t="n">
-        <v>1.44</v>
+        <v>1.404</v>
       </c>
       <c r="J4" t="n">
-        <v>1.46</v>
+        <v>1.41</v>
       </c>
       <c r="K4" t="n">
-        <v>1.388888888888884</v>
+        <v>0.4273504273504258</v>
       </c>
       <c r="L4" t="n">
-        <v>2.388888888888884</v>
+        <v>-0.2726495726495741</v>
       </c>
       <c r="M4" t="n">
-        <v>2.388888888888884</v>
-      </c>
-      <c r="N4" t="b">
-        <v>0</v>
+        <v>0.2726495726495741</v>
+      </c>
+      <c r="N4" t="n">
+        <v>1</v>
       </c>
       <c r="O4" t="inlineStr">
         <is>
@@ -732,19 +732,19 @@
         </is>
       </c>
       <c r="P4" t="n">
-        <v>-0.7414014693577686</v>
+        <v>0.7</v>
       </c>
       <c r="Q4" t="n">
-        <v>2.130290358246652</v>
+        <v>-0.2726495726495741</v>
       </c>
       <c r="R4" t="n">
-        <v>2.130290358246652</v>
-      </c>
-      <c r="S4" t="b">
-        <v>0</v>
+        <v>0.2726495726495741</v>
+      </c>
+      <c r="S4" t="n">
+        <v>1</v>
       </c>
       <c r="T4" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="5">
@@ -764,7 +764,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>ALR</t>
+          <t>AROBS</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -776,25 +776,25 @@
         <v>5</v>
       </c>
       <c r="H5" t="n">
-        <v>0.5</v>
+        <v>-0.3</v>
       </c>
       <c r="I5" t="n">
-        <v>1.51</v>
+        <v>0.679</v>
       </c>
       <c r="J5" t="n">
-        <v>1.505</v>
+        <v>0.67</v>
       </c>
       <c r="K5" t="n">
-        <v>-0.3311258278145823</v>
+        <v>-1.32547864506628</v>
       </c>
       <c r="L5" t="n">
-        <v>-0.8311258278145823</v>
+        <v>-1.02547864506628</v>
       </c>
       <c r="M5" t="n">
-        <v>0.8311258278145823</v>
-      </c>
-      <c r="N5" t="b">
-        <v>0</v>
+        <v>1.02547864506628</v>
+      </c>
+      <c r="N5" t="n">
+        <v>1</v>
       </c>
       <c r="O5" t="inlineStr">
         <is>
@@ -802,19 +802,19 @@
         </is>
       </c>
       <c r="P5" t="n">
-        <v>1.491188456170941</v>
+        <v>-0.3</v>
       </c>
       <c r="Q5" t="n">
-        <v>-1.822314283985524</v>
+        <v>-1.02547864506628</v>
       </c>
       <c r="R5" t="n">
-        <v>1.822314283985524</v>
-      </c>
-      <c r="S5" t="b">
-        <v>0</v>
+        <v>1.02547864506628</v>
+      </c>
+      <c r="S5" t="n">
+        <v>1</v>
       </c>
       <c r="T5" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="6">
@@ -834,36 +834,36 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>AQ</t>
+          <t>BABA</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>RO</t>
+          <t>US</t>
         </is>
       </c>
       <c r="G6" t="n">
         <v>5</v>
       </c>
       <c r="H6" t="n">
-        <v>0.7</v>
+        <v>-0.8</v>
       </c>
       <c r="I6" t="n">
-        <v>1.404</v>
+        <v>158.1300048828125</v>
       </c>
       <c r="J6" t="n">
-        <v>1.41</v>
+        <v>155.6799926757812</v>
       </c>
       <c r="K6" t="n">
-        <v>0.4273504273504258</v>
+        <v>-1.54936579483882</v>
       </c>
       <c r="L6" t="n">
-        <v>-0.2726495726495741</v>
+        <v>-0.7493657948388195</v>
       </c>
       <c r="M6" t="n">
-        <v>0.2726495726495741</v>
-      </c>
-      <c r="N6" t="b">
+        <v>0.7493657948388195</v>
+      </c>
+      <c r="N6" t="n">
         <v>1</v>
       </c>
       <c r="O6" t="inlineStr">
@@ -872,15 +872,15 @@
         </is>
       </c>
       <c r="P6" t="n">
-        <v>1.788867112908102</v>
+        <v>-0.8</v>
       </c>
       <c r="Q6" t="n">
-        <v>-1.361516685557677</v>
+        <v>-0.7493657948388195</v>
       </c>
       <c r="R6" t="n">
-        <v>1.361516685557677</v>
-      </c>
-      <c r="S6" t="b">
+        <v>0.7493657948388195</v>
+      </c>
+      <c r="S6" t="n">
         <v>1</v>
       </c>
       <c r="T6" t="b">
@@ -904,37 +904,37 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>AROBS</t>
+          <t>BATE.DE</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>RO</t>
+          <t>EU</t>
         </is>
       </c>
       <c r="G7" t="n">
         <v>5</v>
       </c>
       <c r="H7" t="n">
-        <v>-0.3</v>
+        <v>0.3</v>
       </c>
       <c r="I7" t="n">
-        <v>0.679</v>
+        <v>24.82999992370605</v>
       </c>
       <c r="J7" t="n">
-        <v>0.67</v>
+        <v>24.69000053405762</v>
       </c>
       <c r="K7" t="n">
-        <v>-1.32547864506628</v>
+        <v>-0.5638316152984379</v>
       </c>
       <c r="L7" t="n">
-        <v>-1.02547864506628</v>
+        <v>-0.863831615298438</v>
       </c>
       <c r="M7" t="n">
-        <v>1.02547864506628</v>
-      </c>
-      <c r="N7" t="b">
-        <v>1</v>
+        <v>0.863831615298438</v>
+      </c>
+      <c r="N7" t="n">
+        <v>0</v>
       </c>
       <c r="O7" t="inlineStr">
         <is>
@@ -942,16 +942,16 @@
         </is>
       </c>
       <c r="P7" t="n">
-        <v>0.3004738292222959</v>
+        <v>0.3</v>
       </c>
       <c r="Q7" t="n">
-        <v>-1.625952474288576</v>
+        <v>-0.863831615298438</v>
       </c>
       <c r="R7" t="n">
-        <v>1.625952474288576</v>
-      </c>
-      <c r="S7" t="b">
-        <v>1</v>
+        <v>0.863831615298438</v>
+      </c>
+      <c r="S7" t="n">
+        <v>0</v>
       </c>
       <c r="T7" t="b">
         <v>0</v>
@@ -1003,7 +1003,7 @@
       <c r="M8" t="n">
         <v>3.912474437627812</v>
       </c>
-      <c r="N8" t="b">
+      <c r="N8" t="n">
         <v>1</v>
       </c>
       <c r="O8" t="inlineStr">
@@ -1012,15 +1012,15 @@
         </is>
       </c>
       <c r="P8" t="n">
-        <v>2.533063754751006</v>
+        <v>1.2</v>
       </c>
       <c r="Q8" t="n">
-        <v>2.579410682876806</v>
+        <v>3.912474437627812</v>
       </c>
       <c r="R8" t="n">
-        <v>2.579410682876806</v>
-      </c>
-      <c r="S8" t="b">
+        <v>3.912474437627812</v>
+      </c>
+      <c r="S8" t="n">
         <v>1</v>
       </c>
       <c r="T8" t="b">
@@ -1073,7 +1073,7 @@
       <c r="M9" t="n">
         <v>5.00095602294456</v>
       </c>
-      <c r="N9" t="b">
+      <c r="N9" t="n">
         <v>1</v>
       </c>
       <c r="O9" t="inlineStr">
@@ -1082,15 +1082,15 @@
         </is>
       </c>
       <c r="P9" t="n">
-        <v>2.979581739856747</v>
+        <v>1.5</v>
       </c>
       <c r="Q9" t="n">
-        <v>3.521374283087812</v>
+        <v>5.00095602294456</v>
       </c>
       <c r="R9" t="n">
-        <v>3.521374283087812</v>
-      </c>
-      <c r="S9" t="b">
+        <v>5.00095602294456</v>
+      </c>
+      <c r="S9" t="n">
         <v>1</v>
       </c>
       <c r="T9" t="b">
@@ -1143,7 +1143,7 @@
       <c r="M10" t="n">
         <v>0.1780346820809301</v>
       </c>
-      <c r="N10" t="b">
+      <c r="N10" t="n">
         <v>1</v>
       </c>
       <c r="O10" t="inlineStr">
@@ -1152,15 +1152,15 @@
         </is>
       </c>
       <c r="P10" t="n">
-        <v>1.34234912780236</v>
+        <v>0.4</v>
       </c>
       <c r="Q10" t="n">
-        <v>-0.7643144457214304</v>
+        <v>0.1780346820809301</v>
       </c>
       <c r="R10" t="n">
-        <v>0.7643144457214304</v>
-      </c>
-      <c r="S10" t="b">
+        <v>0.1780346820809301</v>
+      </c>
+      <c r="S10" t="n">
         <v>1</v>
       </c>
       <c r="T10" t="b">
@@ -1213,7 +1213,7 @@
       <c r="M11" t="n">
         <v>0.01573849878934119</v>
       </c>
-      <c r="N11" t="b">
+      <c r="N11" t="n">
         <v>1</v>
       </c>
       <c r="O11" t="inlineStr">
@@ -1222,15 +1222,15 @@
         </is>
       </c>
       <c r="P11" t="n">
-        <v>1.491188456170941</v>
+        <v>0.5</v>
       </c>
       <c r="Q11" t="n">
-        <v>-1.006926954960282</v>
+        <v>-0.01573849878934119</v>
       </c>
       <c r="R11" t="n">
-        <v>1.006926954960282</v>
-      </c>
-      <c r="S11" t="b">
+        <v>0.01573849878934119</v>
+      </c>
+      <c r="S11" t="n">
         <v>1</v>
       </c>
       <c r="T11" t="b">
@@ -1283,7 +1283,7 @@
       <c r="M12" t="n">
         <v>0.2843137254901933</v>
       </c>
-      <c r="N12" t="b">
+      <c r="N12" t="n">
         <v>1</v>
       </c>
       <c r="O12" t="inlineStr">
@@ -1292,19 +1292,19 @@
         </is>
       </c>
       <c r="P12" t="n">
-        <v>0.002795172485134612</v>
+        <v>-0.5</v>
       </c>
       <c r="Q12" t="n">
-        <v>-0.7871088979753279</v>
+        <v>-0.2843137254901933</v>
       </c>
       <c r="R12" t="n">
-        <v>0.7871088979753279</v>
-      </c>
-      <c r="S12" t="b">
+        <v>0.2843137254901933</v>
+      </c>
+      <c r="S12" t="n">
         <v>1</v>
       </c>
       <c r="T12" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="13">
@@ -1324,37 +1324,37 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>NRF</t>
+          <t>JD</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>RO</t>
+          <t>US</t>
         </is>
       </c>
       <c r="G13" t="n">
         <v>5</v>
       </c>
       <c r="H13" t="n">
-        <v>-1.2</v>
+        <v>-0.5</v>
       </c>
       <c r="I13" t="n">
-        <v>2.71</v>
+        <v>29.92000007629395</v>
       </c>
       <c r="J13" t="n">
-        <v>2.72</v>
+        <v>29.44000053405762</v>
       </c>
       <c r="K13" t="n">
-        <v>0.3690036900369176</v>
+        <v>-1.604276540816718</v>
       </c>
       <c r="L13" t="n">
-        <v>1.569003690036918</v>
+        <v>-1.104276540816718</v>
       </c>
       <c r="M13" t="n">
-        <v>1.569003690036918</v>
-      </c>
-      <c r="N13" t="b">
-        <v>0</v>
+        <v>1.104276540816718</v>
+      </c>
+      <c r="N13" t="n">
+        <v>1</v>
       </c>
       <c r="O13" t="inlineStr">
         <is>
@@ -1362,19 +1362,19 @@
         </is>
       </c>
       <c r="P13" t="n">
-        <v>-1.03908012609493</v>
+        <v>-0.5</v>
       </c>
       <c r="Q13" t="n">
-        <v>1.408083816131847</v>
+        <v>-1.104276540816718</v>
       </c>
       <c r="R13" t="n">
-        <v>1.408083816131847</v>
-      </c>
-      <c r="S13" t="b">
-        <v>0</v>
+        <v>1.104276540816718</v>
+      </c>
+      <c r="S13" t="n">
+        <v>1</v>
       </c>
       <c r="T13" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="14">
@@ -1394,37 +1394,37 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>SNN</t>
+          <t>LHA.DE</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>RO</t>
+          <t>EU</t>
         </is>
       </c>
       <c r="G14" t="n">
         <v>5</v>
       </c>
       <c r="H14" t="n">
-        <v>1</v>
+        <v>-0.4</v>
       </c>
       <c r="I14" t="n">
-        <v>52</v>
+        <v>8.255999565124512</v>
       </c>
       <c r="J14" t="n">
-        <v>54.8</v>
+        <v>8.465999603271484</v>
       </c>
       <c r="K14" t="n">
-        <v>5.384615384615388</v>
+        <v>2.543605247195835</v>
       </c>
       <c r="L14" t="n">
-        <v>4.384615384615388</v>
+        <v>2.943605247195835</v>
       </c>
       <c r="M14" t="n">
-        <v>4.384615384615388</v>
-      </c>
-      <c r="N14" t="b">
-        <v>1</v>
+        <v>2.943605247195835</v>
+      </c>
+      <c r="N14" t="n">
+        <v>0</v>
       </c>
       <c r="O14" t="inlineStr">
         <is>
@@ -1432,19 +1432,19 @@
         </is>
       </c>
       <c r="P14" t="n">
-        <v>2.235385098013844</v>
+        <v>-0.4</v>
       </c>
       <c r="Q14" t="n">
-        <v>3.149230286601544</v>
+        <v>2.943605247195835</v>
       </c>
       <c r="R14" t="n">
-        <v>3.149230286601544</v>
-      </c>
-      <c r="S14" t="b">
-        <v>1</v>
+        <v>2.943605247195835</v>
+      </c>
+      <c r="S14" t="n">
+        <v>0</v>
       </c>
       <c r="T14" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="15">
@@ -1464,36 +1464,36 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>SNP</t>
+          <t>NIO</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>RO</t>
+          <t>US</t>
         </is>
       </c>
       <c r="G15" t="n">
         <v>5</v>
       </c>
       <c r="H15" t="n">
-        <v>0.6</v>
+        <v>-1</v>
       </c>
       <c r="I15" t="n">
-        <v>0.9645</v>
+        <v>5.099999904632568</v>
       </c>
       <c r="J15" t="n">
-        <v>0.9735</v>
+        <v>5.03000020980835</v>
       </c>
       <c r="K15" t="n">
-        <v>0.9331259720062324</v>
+        <v>-1.372543061434861</v>
       </c>
       <c r="L15" t="n">
-        <v>0.3331259720062324</v>
+        <v>-0.372543061434861</v>
       </c>
       <c r="M15" t="n">
-        <v>0.3331259720062324</v>
-      </c>
-      <c r="N15" t="b">
+        <v>0.372543061434861</v>
+      </c>
+      <c r="N15" t="n">
         <v>1</v>
       </c>
       <c r="O15" t="inlineStr">
@@ -1502,15 +1502,15 @@
         </is>
       </c>
       <c r="P15" t="n">
-        <v>1.640027784539522</v>
+        <v>-1</v>
       </c>
       <c r="Q15" t="n">
-        <v>-0.7069018125332893</v>
+        <v>-0.372543061434861</v>
       </c>
       <c r="R15" t="n">
-        <v>0.7069018125332893</v>
-      </c>
-      <c r="S15" t="b">
+        <v>0.372543061434861</v>
+      </c>
+      <c r="S15" t="n">
         <v>1</v>
       </c>
       <c r="T15" t="b">
@@ -1534,7 +1534,7 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>TLV</t>
+          <t>NRF</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -1546,25 +1546,25 @@
         <v>5</v>
       </c>
       <c r="H16" t="n">
-        <v>0.7</v>
+        <v>-1.2</v>
       </c>
       <c r="I16" t="n">
-        <v>29.98</v>
+        <v>2.71</v>
       </c>
       <c r="J16" t="n">
-        <v>30.28</v>
+        <v>2.72</v>
       </c>
       <c r="K16" t="n">
-        <v>1.000667111407605</v>
+        <v>0.3690036900369176</v>
       </c>
       <c r="L16" t="n">
-        <v>0.3006671114076049</v>
+        <v>1.569003690036918</v>
       </c>
       <c r="M16" t="n">
-        <v>0.3006671114076049</v>
-      </c>
-      <c r="N16" t="b">
-        <v>1</v>
+        <v>1.569003690036918</v>
+      </c>
+      <c r="N16" t="n">
+        <v>0</v>
       </c>
       <c r="O16" t="inlineStr">
         <is>
@@ -1572,19 +1572,19 @@
         </is>
       </c>
       <c r="P16" t="n">
-        <v>1.788867112908102</v>
+        <v>-1.2</v>
       </c>
       <c r="Q16" t="n">
-        <v>-0.7882000015004975</v>
+        <v>1.569003690036918</v>
       </c>
       <c r="R16" t="n">
-        <v>0.7882000015004975</v>
-      </c>
-      <c r="S16" t="b">
-        <v>1</v>
+        <v>1.569003690036918</v>
+      </c>
+      <c r="S16" t="n">
+        <v>0</v>
       </c>
       <c r="T16" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="17">
@@ -1604,36 +1604,36 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>TRP</t>
+          <t>PATH</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>RO</t>
+          <t>US</t>
         </is>
       </c>
       <c r="G17" t="n">
         <v>5</v>
       </c>
       <c r="H17" t="n">
-        <v>0.8</v>
+        <v>2.5</v>
       </c>
       <c r="I17" t="n">
-        <v>0.442</v>
+        <v>19.29000091552734</v>
       </c>
       <c r="J17" t="n">
-        <v>0.4405</v>
+        <v>17.42000007629395</v>
       </c>
       <c r="K17" t="n">
-        <v>-0.3393665158371029</v>
+        <v>-9.694145933026654</v>
       </c>
       <c r="L17" t="n">
-        <v>-1.139366515837103</v>
+        <v>-12.19414593302665</v>
       </c>
       <c r="M17" t="n">
-        <v>1.139366515837103</v>
-      </c>
-      <c r="N17" t="b">
+        <v>12.19414593302665</v>
+      </c>
+      <c r="N17" t="n">
         <v>0</v>
       </c>
       <c r="O17" t="inlineStr">
@@ -1642,15 +1642,15 @@
         </is>
       </c>
       <c r="P17" t="n">
-        <v>1.937706441276683</v>
+        <v>2.5</v>
       </c>
       <c r="Q17" t="n">
-        <v>-2.277072957113786</v>
+        <v>-12.19414593302665</v>
       </c>
       <c r="R17" t="n">
-        <v>2.277072957113786</v>
-      </c>
-      <c r="S17" t="b">
+        <v>12.19414593302665</v>
+      </c>
+      <c r="S17" t="n">
         <v>0</v>
       </c>
       <c r="T17" t="b">
@@ -1674,7 +1674,7 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>WINE</t>
+          <t>SNN</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -1686,25 +1686,25 @@
         <v>5</v>
       </c>
       <c r="H18" t="n">
-        <v>0.8</v>
+        <v>1</v>
       </c>
       <c r="I18" t="n">
-        <v>18.72</v>
+        <v>52</v>
       </c>
       <c r="J18" t="n">
-        <v>18.56</v>
+        <v>54.8</v>
       </c>
       <c r="K18" t="n">
-        <v>-0.8547008547008517</v>
+        <v>5.384615384615388</v>
       </c>
       <c r="L18" t="n">
-        <v>-1.654700854700852</v>
+        <v>4.384615384615388</v>
       </c>
       <c r="M18" t="n">
-        <v>1.654700854700852</v>
-      </c>
-      <c r="N18" t="b">
-        <v>0</v>
+        <v>4.384615384615388</v>
+      </c>
+      <c r="N18" t="n">
+        <v>1</v>
       </c>
       <c r="O18" t="inlineStr">
         <is>
@@ -1712,19 +1712,19 @@
         </is>
       </c>
       <c r="P18" t="n">
-        <v>1.937706441276683</v>
+        <v>1</v>
       </c>
       <c r="Q18" t="n">
-        <v>-2.792407295977535</v>
+        <v>4.384615384615388</v>
       </c>
       <c r="R18" t="n">
-        <v>2.792407295977535</v>
-      </c>
-      <c r="S18" t="b">
-        <v>0</v>
+        <v>4.384615384615388</v>
+      </c>
+      <c r="S18" t="n">
+        <v>1</v>
       </c>
       <c r="T18" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="19">
@@ -1744,36 +1744,36 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>BABA</t>
+          <t>SNP</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>RO</t>
         </is>
       </c>
       <c r="G19" t="n">
         <v>5</v>
       </c>
       <c r="H19" t="n">
-        <v>-0.8</v>
+        <v>0.6</v>
       </c>
       <c r="I19" t="n">
-        <v>158.1300048828125</v>
+        <v>0.9645</v>
       </c>
       <c r="J19" t="n">
-        <v>155.6799926757812</v>
+        <v>0.9735</v>
       </c>
       <c r="K19" t="n">
-        <v>-1.54936579483882</v>
+        <v>0.9331259720062324</v>
       </c>
       <c r="L19" t="n">
-        <v>-0.7493657948388195</v>
+        <v>0.3331259720062324</v>
       </c>
       <c r="M19" t="n">
-        <v>0.7493657948388195</v>
-      </c>
-      <c r="N19" t="b">
+        <v>0.3331259720062324</v>
+      </c>
+      <c r="N19" t="n">
         <v>1</v>
       </c>
       <c r="O19" t="inlineStr">
@@ -1782,15 +1782,15 @@
         </is>
       </c>
       <c r="P19" t="n">
-        <v>-0.01896517362332979</v>
+        <v>0.6</v>
       </c>
       <c r="Q19" t="n">
-        <v>-1.53040062121549</v>
+        <v>0.3331259720062324</v>
       </c>
       <c r="R19" t="n">
-        <v>1.53040062121549</v>
-      </c>
-      <c r="S19" t="b">
+        <v>0.3331259720062324</v>
+      </c>
+      <c r="S19" t="n">
         <v>1</v>
       </c>
       <c r="T19" t="b">
@@ -1814,36 +1814,36 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>JD</t>
+          <t>TLV</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>RO</t>
         </is>
       </c>
       <c r="G20" t="n">
         <v>5</v>
       </c>
       <c r="H20" t="n">
-        <v>-0.5</v>
+        <v>0.7</v>
       </c>
       <c r="I20" t="n">
-        <v>29.92000007629395</v>
+        <v>29.98</v>
       </c>
       <c r="J20" t="n">
-        <v>29.44000053405762</v>
+        <v>30.28</v>
       </c>
       <c r="K20" t="n">
-        <v>-1.604276540816718</v>
+        <v>1.000667111407605</v>
       </c>
       <c r="L20" t="n">
-        <v>-1.104276540816718</v>
+        <v>0.3006671114076049</v>
       </c>
       <c r="M20" t="n">
-        <v>1.104276540816718</v>
-      </c>
-      <c r="N20" t="b">
+        <v>0.3006671114076049</v>
+      </c>
+      <c r="N20" t="n">
         <v>1</v>
       </c>
       <c r="O20" t="inlineStr">
@@ -1852,19 +1852,19 @@
         </is>
       </c>
       <c r="P20" t="n">
-        <v>0.168737664365881</v>
+        <v>0.7</v>
       </c>
       <c r="Q20" t="n">
-        <v>-1.773014205182599</v>
+        <v>0.3006671114076049</v>
       </c>
       <c r="R20" t="n">
-        <v>1.773014205182599</v>
-      </c>
-      <c r="S20" t="b">
+        <v>0.3006671114076049</v>
+      </c>
+      <c r="S20" t="n">
         <v>1</v>
       </c>
       <c r="T20" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="21">
@@ -1884,37 +1884,37 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>NIO</t>
+          <t>TRP</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>RO</t>
         </is>
       </c>
       <c r="G21" t="n">
         <v>5</v>
       </c>
       <c r="H21" t="n">
-        <v>-1</v>
+        <v>0.8</v>
       </c>
       <c r="I21" t="n">
-        <v>5.099999904632568</v>
+        <v>0.442</v>
       </c>
       <c r="J21" t="n">
-        <v>5.03000020980835</v>
+        <v>0.4405</v>
       </c>
       <c r="K21" t="n">
-        <v>-1.372543061434861</v>
+        <v>-0.3393665158371029</v>
       </c>
       <c r="L21" t="n">
-        <v>-0.372543061434861</v>
+        <v>-1.139366515837103</v>
       </c>
       <c r="M21" t="n">
-        <v>0.372543061434861</v>
-      </c>
-      <c r="N21" t="b">
-        <v>1</v>
+        <v>1.139366515837103</v>
+      </c>
+      <c r="N21" t="n">
+        <v>0</v>
       </c>
       <c r="O21" t="inlineStr">
         <is>
@@ -1922,19 +1922,19 @@
         </is>
       </c>
       <c r="P21" t="n">
-        <v>-0.1441003989494702</v>
+        <v>0.8</v>
       </c>
       <c r="Q21" t="n">
-        <v>-1.228442662485391</v>
+        <v>-1.139366515837103</v>
       </c>
       <c r="R21" t="n">
-        <v>1.228442662485391</v>
-      </c>
-      <c r="S21" t="b">
-        <v>1</v>
+        <v>1.139366515837103</v>
+      </c>
+      <c r="S21" t="n">
+        <v>0</v>
       </c>
       <c r="T21" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="22">
@@ -1954,36 +1954,36 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>PATH</t>
+          <t>WINE</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>RO</t>
         </is>
       </c>
       <c r="G22" t="n">
         <v>5</v>
       </c>
       <c r="H22" t="n">
-        <v>2.5</v>
+        <v>0.8</v>
       </c>
       <c r="I22" t="n">
-        <v>19.29000091552734</v>
+        <v>18.72</v>
       </c>
       <c r="J22" t="n">
-        <v>17.42000007629395</v>
+        <v>18.56</v>
       </c>
       <c r="K22" t="n">
-        <v>-9.694145933026654</v>
+        <v>-0.8547008547008517</v>
       </c>
       <c r="L22" t="n">
-        <v>-12.19414593302665</v>
+        <v>-1.654700854700852</v>
       </c>
       <c r="M22" t="n">
-        <v>12.19414593302665</v>
-      </c>
-      <c r="N22" t="b">
+        <v>1.654700854700852</v>
+      </c>
+      <c r="N22" t="n">
         <v>0</v>
       </c>
       <c r="O22" t="inlineStr">
@@ -1992,15 +1992,15 @@
         </is>
       </c>
       <c r="P22" t="n">
-        <v>2.045766044257989</v>
+        <v>0.8</v>
       </c>
       <c r="Q22" t="n">
-        <v>-11.73991197728464</v>
+        <v>-1.654700854700852</v>
       </c>
       <c r="R22" t="n">
-        <v>11.73991197728464</v>
-      </c>
-      <c r="S22" t="b">
+        <v>1.654700854700852</v>
+      </c>
+      <c r="S22" t="n">
         <v>0</v>
       </c>
       <c r="T22" t="b">
@@ -2111,7 +2111,7 @@
         <v>15</v>
       </c>
       <c r="E3" t="n">
-        <v>66.66666666666666</v>
+        <v>0.6666666666666666</v>
       </c>
       <c r="F3" t="n">
         <v>1.552742655330417</v>
@@ -2141,7 +2141,7 @@
         <v>4</v>
       </c>
       <c r="E4" t="n">
-        <v>75</v>
+        <v>0.75</v>
       </c>
       <c r="F4" t="n">
         <v>3.605082832529263</v>
@@ -2202,13 +2202,13 @@
         <v>61.90476190476191</v>
       </c>
       <c r="C2" t="n">
-        <v>52.38095238095239</v>
+        <v>61.90476190476191</v>
       </c>
       <c r="D2" t="n">
         <v>1.977090858217504</v>
       </c>
       <c r="E2" t="n">
-        <v>2.204949757316726</v>
+        <v>1.977090858217504</v>
       </c>
     </row>
   </sheetData>
@@ -2222,7 +2222,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2"/>
+  <dimension ref="A1:C2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2238,11 +2238,6 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>model_version_tag</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
           <t>notes</t>
         </is>
       </c>
@@ -2253,17 +2248,12 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>{'EU': {'alpha': 1.1987554948212646, 'beta': -1.363650769379695, 'mae': 1.5399801618904165, 'n': 4}, 'RO': {'alpha': 0.7469918143280379, 'beta': 1.4883932836858065, 'mae': 1.8666532416497092, 'n': 30}, 'US': {'alpha': 1.5049241490038507, 'beta': 0.45523789572094536, 'mae': 7.088996103187562, 'n': 8}}</t>
+          <t>{'RO': {'mult': 1.0, 'bias': 0.0, 'clip_pct': 6.0}, 'EU': {'mult': 1.0, 'bias': 0.0, 'clip_pct': 6.0}, 'US': {'mult': 1.0, 'bias': 0.0, 'clip_pct': 6.0}}</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>StockD_V10.7F+</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>region-level linear calibration (winsorized)</t>
+          <t>bootstrap</t>
         </is>
       </c>
     </row>

</xml_diff>